<commit_message>
Update sample Excel for clearer import demo
</commit_message>
<xml_diff>
--- a/samples/sample_tasks.xlsx
+++ b/samples/sample_tasks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,42 +446,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Discovery</t>
+          <t>Сбор требований</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Clarify goals and constraints</t>
+          <t>Уточнить цели, ограничения и формат результата.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PM</t>
+          <t>Аналитик</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Plan MVP</t>
+          <t>UX-макет</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Create simple task plan</t>
+          <t>Подготовить экран Гантта, чат и модалку.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Planner</t>
+          <t>Дизайнер</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -492,50 +492,75 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Implement demo</t>
+          <t>Backend API</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Build import, chart, chat, and export flow</t>
+          <t>Сделать импорт, экспорт и чат-команды.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Stakeholder review</t>
+          <t>Frontend UI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Review generated plan and export</t>
+          <t>Собрать интерфейс и связать его с API.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>T2,T3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Демо заказчику</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Показать сценарий и собрать обратную связь.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Заказчик</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
         <v>1</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>T3</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>T4</t>
         </is>
       </c>
     </row>

</xml_diff>